<commit_message>
Refresh aquaculture outputs and dashboard sales filters
</commit_message>
<xml_diff>
--- a/output/freshwater/Europe_freshwater_summary_latest.xlsx
+++ b/output/freshwater/Europe_freshwater_summary_latest.xlsx
@@ -4780,7 +4780,7 @@
         <v>2021</v>
       </c>
       <c r="C184" t="n">
-        <v>22278</v>
+        <v>445</v>
       </c>
       <c r="D184" t="n">
         <v>11303</v>
@@ -4789,7 +4789,7 @@
         <v>93</v>
       </c>
       <c r="F184" t="n">
-        <v>611051</v>
+        <v>2961228</v>
       </c>
       <c r="G184" t="n">
         <v>39880458</v>
@@ -4806,7 +4806,7 @@
         <v>2022</v>
       </c>
       <c r="C185" t="n">
-        <v>0</v>
+        <v>566</v>
       </c>
       <c r="D185" t="n">
         <v>8981</v>
@@ -4815,7 +4815,7 @@
         <v>1431</v>
       </c>
       <c r="F185" t="n">
-        <v>0</v>
+        <v>3019676</v>
       </c>
       <c r="G185" t="n">
         <v>55032205</v>
@@ -4832,7 +4832,7 @@
         <v>2023</v>
       </c>
       <c r="C186" t="n">
-        <v>52</v>
+        <v>548</v>
       </c>
       <c r="D186" t="n">
         <v>9154</v>
@@ -4841,7 +4841,7 @@
         <v>1274</v>
       </c>
       <c r="F186" t="n">
-        <v>511900</v>
+        <v>3113485</v>
       </c>
       <c r="G186" t="n">
         <v>43024287</v>
@@ -4858,12 +4858,12 @@
         <v>2024</v>
       </c>
       <c r="C187" t="n">
-        <v>8176</v>
+        <v>745</v>
       </c>
       <c r="D187"/>
       <c r="E187"/>
       <c r="F187" t="n">
-        <v>40125428</v>
+        <v>4003542</v>
       </c>
       <c r="G187"/>
       <c r="H187"/>

</xml_diff>